<commit_message>
Commiting BaseTest, ArrayTest, ArrayPage, Helper, HomePage, config.properties, TestDataSheet
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/TestDataSheet.xlsx
+++ b/src/test/resources/testData/TestDataSheet.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\god\eclipse-workspace\DS-AlgoProj\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8726EDC4-9EE6-4A66-887B-6D65BCF411A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D6B520-4BDB-4782-8EA3-448B9ED3EEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="371" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="371" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginSheet" sheetId="1" r:id="rId1"/>
     <sheet name="pythonCode" sheetId="2" r:id="rId2"/>
-    <sheet name="Practice Questions" sheetId="3" r:id="rId3"/>
+    <sheet name="PracticeQuestions" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="16">
   <si>
     <t>Vijayabharathi</t>
   </si>
@@ -58,70 +58,6 @@
   </si>
   <si>
     <t>hello</t>
-  </si>
-  <si>
-    <t>def search(input_list, num):
-if(num in input_list):
-print("Element Found")
-\b
-\b
-else:
-print("Not Found")
-\b
-\b
-\b
-\b
-search([12, 23, 45, 67, 6, 90] , 12)</t>
-  </si>
-  <si>
-    <t>def findMaxConsecutiveOnes(nums) :
-count = 0
-result = 0
-for i in range(0, len(nums)):
-if (nums[i] == 0):
-count = 0
-\b
-\b
-else:
-count+= 1
-\b
-\b
-result = max(result, count)
-\b
-\b
-print(result)
-\b
-\b
-findMaxConsecutiveOnes([1,0,1,1,0,1])</t>
-  </si>
-  <si>
-    <t>def findNumbers(nums):
-c=0
-for i in nums:
-j=str(i)
-x=len(j)
-if x%2==0:
-c=c+1
-\b
-\b
-\b
-\b
-print c
-return c
-findNumbers([12,345,2,6,7896])</t>
-  </si>
-  <si>
-    <t>def sortedSquares(nums):
-squares_list = []
-for i in range(0, len(nums)):
-square = nums[i] * nums[i];
-squares_list.append(square)
-\b
-\b
-sorted_squares_list = sorted(squares_list)
-print sorted_squares_list;
-return sorted_squares_list;
-sortedSquares([-7,-3,2,3,11])</t>
   </si>
   <si>
     <t>TC002</t>
@@ -140,7 +76,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -167,29 +103,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -205,17 +130,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="17" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,7 +534,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>11</v>
@@ -620,44 +542,44 @@
       <c r="C3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>19</v>
+      <c r="D3" s="6" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="6"/>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="6"/>
+      <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="6"/>
+      <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D8" s="6"/>
+      <c r="D8" s="5"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" s="6"/>
+      <c r="D9" s="5"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D10" s="6"/>
+      <c r="D10" s="5"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D11" s="6"/>
+      <c r="D11" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -666,7 +588,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BB2F416-0080-4CD5-8640-78BD573AE583}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -693,64 +615,24 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>19</v>
+      <c r="C3" s="6" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>